<commit_message>
Fix SAML metadata: remove >4096-char CFN param, inline placeholder provider, apply real XML via update-saml-provider
</commit_message>
<xml_diff>
--- a/deliverables/AWS-Infrastructure-Resource-Inventory.xlsx
+++ b/deliverables/AWS-Infrastructure-Resource-Inventory.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resource Inventory'!$A$1:$G$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parameters'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parameters'!$A$1:$D$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Conditions'!$A$1:$C$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Outputs'!$A$1:$C$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'VPN Config'!$A$1:$D$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'VPN Config'!$A$1:$D$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Users &amp; Permissions'!$A$1:$D$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2607,7 +2607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2949,7 +2949,7 @@
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>SamlMetadataDocument</t>
+          <t>SplitTunnel</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -2959,39 +2959,17 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>(placeholder XML)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Entra ID federation metadata</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="17" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t>SplitTunnel</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
           <t>true / false</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D17"/>
+  <autoFilter ref="A1:D16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -3441,7 +3419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3701,42 +3679,46 @@
     <row r="13" ht="29" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>Site-to-Site</t>
+          <t>SAML metadata</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Customer gateway</t>
+          <t>How it is applied</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>ipsec.1 · ASN 65000</t>
+          <t>Out-of-band: aws iam update-saml-provider</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Conditional</t>
+          <t>Real Entra ID XML is ~13 KB — too large for a CFN String param (4096 limit); template carries a placeholder provider</t>
         </is>
       </c>
     </row>
     <row r="14" ht="29" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>Site-to-Site</t>
+          <t>SAML metadata</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Routing</t>
+          <t>Post-deploy command</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Static · prop. to pri/db RTs</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr"/>
+          <t>update-saml-provider --saml-provider-arn &lt;output&gt; --saml-metadata-document file://&lt;xml&gt;</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Before anyone can SSO in</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="29" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
@@ -3746,22 +3728,62 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
+          <t>Customer gateway</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>ipsec.1 · ASN 65000</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Conditional</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="29" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Site-to-Site</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Routing</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Static · prop. to pri/db RTs</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17" ht="29" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Site-to-Site</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
           <t>Tunnel config</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>VPC console → download configuration</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Share with on-prem team</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D15"/>
+  <autoFilter ref="A1:D17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix ClientVpnEndpoint VpcId (SG requires VPC), retain flow-log bucket on delete
</commit_message>
<xml_diff>
--- a/deliverables/AWS-Infrastructure-Resource-Inventory.xlsx
+++ b/deliverables/AWS-Infrastructure-Resource-Inventory.xlsx
@@ -1338,7 +1338,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>SSE-S3 · lifecycle: Glacier @30d · expire @365d</t>
+          <t>SSE-S3 · lifecycle: Glacier @30d · expire @365d · DeletionPolicy: Retain</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>VPC flow logs</t>
+          <t>VPC flow logs — retained on stack delete (empty manually)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove VPC flow logs: drop FlowLogBucket + VpcFlowLog from template and all deliverables
- Template: delete S3 bucket and flow log resources, keep template lint-clean
- README: drop flow-log rows/bullets, cfn-guard findings now 9 (was 14)
- Deliverables: remove flow-log chips/bullets/rows from PPTX, EXCEL, DOCX
- Doc generator regenerated
</commit_message>
<xml_diff>
--- a/deliverables/AWS-Infrastructure-Resource-Inventory.xlsx
+++ b/deliverables/AWS-Infrastructure-Resource-Inventory.xlsx
@@ -16,10 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users &amp; Permissions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resource Inventory'!$A$1:$G$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resource Inventory'!$A$1:$G$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parameters'!$A$1:$D$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Conditions'!$A$1:$C$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Outputs'!$A$1:$C$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Outputs'!$A$1:$C$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'VPN Config'!$A$1:$D$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Users &amp; Permissions'!$A$1:$D$5</definedName>
   </definedNames>
@@ -714,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1323,22 +1323,22 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>FlowLogBucket</t>
+          <t>PubSubnetARouteAssoc</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>AWS::S3::Bucket</t>
+          <t>AWS::EC2::SubnetRouteTableAssociation</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-flowlog-&lt;acct&gt;</t>
+          <t>pub-a → pub rtb</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>SSE-S3 · lifecycle: Glacier @30d · expire @365d · DeletionPolicy: Retain</t>
+          <t>Association</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1346,11 +1346,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>VPC flow logs — retained on stack delete (empty manually)</t>
-        </is>
-      </c>
+      <c r="G18" s="8" t="inlineStr"/>
     </row>
     <row r="19" ht="43.5" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -1360,22 +1356,22 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>VpcFlowLog</t>
+          <t>PubSubnetCRouteAssoc</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::FlowLog</t>
+          <t>AWS::EC2::SubnetRouteTableAssociation</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>VPC flow log</t>
+          <t>pub-c → pub rtb</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>ALL traffic → S3 · 10 min aggregation</t>
+          <t>Association</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
@@ -1393,7 +1389,7 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>PubSubnetARouteAssoc</t>
+          <t>PriSubnetARouteAssoc</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
@@ -1403,7 +1399,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>pub-a → pub rtb</t>
+          <t>pri-a → pri rtb</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1426,7 +1422,7 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>PubSubnetCRouteAssoc</t>
+          <t>PriSubnetCRouteAssoc</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -1436,7 +1432,7 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>pub-c → pub rtb</t>
+          <t>pri-c → pri rtb</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -1459,7 +1455,7 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>PriSubnetARouteAssoc</t>
+          <t>DbSubnetARouteAssoc</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
@@ -1469,7 +1465,7 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>pri-a → pri rtb</t>
+          <t>db-a → db rtb</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -1492,7 +1488,7 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>PriSubnetCRouteAssoc</t>
+          <t>DbSubnetCRouteAssoc</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -1502,7 +1498,7 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>pri-c → pri rtb</t>
+          <t>db-c → db rtb</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -1518,29 +1514,29 @@
       <c r="G23" s="10" t="inlineStr"/>
     </row>
     <row r="24" ht="43.5" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Network</t>
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Security</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>DbSubnetARouteAssoc</t>
+          <t>CommonSg</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::SubnetRouteTableAssociation</t>
+          <t>AWS::EC2::SecurityGroup</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>db-a → db rtb</t>
+          <t>hmsg-rac-prd-common-ec2-sg-ec1</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Association</t>
+          <t>RDP 3389 ← 10.200.0.0/22 · egress 443 → VPC</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1548,32 +1544,36 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Windows admin</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="43.5" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>Network</t>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Security</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>DbSubnetCRouteAssoc</t>
+          <t>MssqlSg</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::SubnetRouteTableAssociation</t>
+          <t>AWS::EC2::SecurityGroup</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>db-c → db rtb</t>
+          <t>hmsg-rac-prd-mssql-ec2-sg-ec1</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Association</t>
+          <t>MSSQL 1433 ← 10.200.0.0/22 · egress 443 → VPC</t>
         </is>
       </c>
       <c r="F25" s="10" t="inlineStr">
@@ -1581,7 +1581,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G25" s="10" t="inlineStr"/>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>SQL access</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="43.5" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
@@ -1591,34 +1595,30 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>CommonSg</t>
+          <t>CommonSgOnPremRdp</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::SecurityGroup</t>
+          <t>AWS::EC2::SecurityGroupIngress</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-common-ec2-sg-ec1</t>
+          <t>RDP from on-prem</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>RDP 3389 ← 10.200.0.0/22 · egress 443 → VPC</t>
+          <t>3389 ← OnPremCidr</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>Windows admin</t>
-        </is>
-      </c>
+          <t>CreateSiteToSiteVpn</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr"/>
     </row>
     <row r="27" ht="43.5" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
@@ -1628,34 +1628,30 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>MssqlSg</t>
+          <t>MssqlSgOnPremMssql</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::SecurityGroup</t>
+          <t>AWS::EC2::SecurityGroupIngress</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-mssql-ec2-sg-ec1</t>
+          <t>MSSQL from on-prem</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>MSSQL 1433 ← 10.200.0.0/22 · egress 443 → VPC</t>
+          <t>1433 ← OnPremCidr</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G27" s="10" t="inlineStr">
-        <is>
-          <t>SQL access</t>
-        </is>
-      </c>
+          <t>CreateSiteToSiteVpn</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr"/>
     </row>
     <row r="28" ht="43.5" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
@@ -1665,30 +1661,34 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>CommonSgOnPremRdp</t>
+          <t>ClientVpnSg</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::SecurityGroupIngress</t>
+          <t>AWS::EC2::SecurityGroup</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>RDP from on-prem</t>
+          <t>hmsg-rac-prd-clientvpn-sg-ec1</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>3389 ← OnPremCidr</t>
+          <t>UDP 443 ← 0.0.0.0/0 · egress 3389/1433 → VPC</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>CreateSiteToSiteVpn</t>
-        </is>
-      </c>
-      <c r="G28" s="8" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Endpoint SG</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="43.5" customHeight="1">
       <c r="A29" s="12" t="inlineStr">
@@ -1698,55 +1698,59 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>MssqlSgOnPremMssql</t>
+          <t>VpcEndpointSg</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::SecurityGroupIngress</t>
+          <t>AWS::EC2::SecurityGroup</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>MSSQL from on-prem</t>
+          <t>hmsg-rac-prd-vpce-sg-ec1</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>1433 ← OnPremCidr</t>
+          <t>TCP 443 ← VPC CIDR</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>CreateSiteToSiteVpn</t>
-        </is>
-      </c>
-      <c r="G29" s="10" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>Interface endpoints</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="43.5" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>Security</t>
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Compute</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>ClientVpnSg</t>
+          <t>SysadmSecret</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::SecurityGroup</t>
+          <t>AWS::SecretsManager::Secret</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-clientvpn-sg-ec1</t>
+          <t>hmsg-rac-prd-sysadm-password</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>UDP 443 ← 0.0.0.0/0 · egress 3389/1433 → VPC</t>
+          <t>sysadm password (NoEcho) · retained</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -1754,36 +1758,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>Endpoint SG</t>
-        </is>
-      </c>
+      <c r="G30" s="8" t="inlineStr"/>
     </row>
     <row r="31" ht="43.5" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>Security</t>
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Compute</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>VpcEndpointSg</t>
+          <t>Ec2Role</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::SecurityGroup</t>
+          <t>AWS::IAM::Role</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-vpce-sg-ec1</t>
+          <t>EC2 instance role</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>TCP 443 ← VPC CIDR</t>
+          <t>AmazonSSMManagedInstanceCore · GetSecretValue (1 secret)</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr">
@@ -1791,11 +1791,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G31" s="10" t="inlineStr">
-        <is>
-          <t>Interface endpoints</t>
-        </is>
-      </c>
+      <c r="G31" s="10" t="inlineStr"/>
     </row>
     <row r="32" ht="43.5" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
@@ -1805,22 +1801,22 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>SysadmSecret</t>
+          <t>Ec2InstanceProfile</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>AWS::SecretsManager::Secret</t>
+          <t>AWS::IAM::InstanceProfile</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-sysadm-password</t>
+          <t>EC2 instance profile</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>sysadm password (NoEcho) · retained</t>
+          <t>Attaches Ec2Role</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -1838,22 +1834,22 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Ec2Role</t>
+          <t>MssqlInstance</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>AWS::IAM::Role</t>
+          <t>AWS::EC2::Instance</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>EC2 instance role</t>
+          <t>hmsg-rac-prd-mssql01-ec2-ec1a</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>AmazonSSMManagedInstanceCore · GetSecretValue (1 secret)</t>
+          <t>m7i.2xlarge · Win 2022 EN · 250 GB root + 4 TB D: · IMDSv2</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
@@ -1861,7 +1857,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G33" s="10" t="inlineStr"/>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>EB S-optimised · retained</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="43.5" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
@@ -1871,22 +1871,22 @@
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Ec2InstanceProfile</t>
+          <t>SecretsManagerEndpoint</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>AWS::IAM::InstanceProfile</t>
+          <t>AWS::EC2::VPCEndpoint</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>EC2 instance profile</t>
+          <t>com.amazonaws.eu-central-1.secretsmanager</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Attaches Ec2Role</t>
+          <t>Interface · DbSubnetA · private DNS</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -1904,22 +1904,22 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>MssqlInstance</t>
+          <t>SsmEndpoint</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::Instance</t>
+          <t>AWS::EC2::VPCEndpoint</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-mssql01-ec2-ec1a</t>
+          <t>com.amazonaws.eu-central-1.ssm</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>m7i.2xlarge · Win 2022 EN · 250 GB root + 4 TB D: · IMDSv2</t>
+          <t>Interface · DbSubnetA · private DNS</t>
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr">
@@ -1927,11 +1927,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G35" s="10" t="inlineStr">
-        <is>
-          <t>EB S-optimised · retained</t>
-        </is>
-      </c>
+      <c r="G35" s="10" t="inlineStr"/>
     </row>
     <row r="36" ht="43.5" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
@@ -1941,7 +1937,7 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>SecretsManagerEndpoint</t>
+          <t>SsmMessagesEndpoint</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
@@ -1951,7 +1947,7 @@
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>com.amazonaws.eu-central-1.secretsmanager</t>
+          <t>com.amazonaws.eu-central-1.ssmmessages</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
@@ -1974,7 +1970,7 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>SsmEndpoint</t>
+          <t>Ec2MessagesEndpoint</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
@@ -1984,7 +1980,7 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>com.amazonaws.eu-central-1.ssm</t>
+          <t>com.amazonaws.eu-central-1.ec2messages</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -2000,29 +1996,29 @@
       <c r="G37" s="10" t="inlineStr"/>
     </row>
     <row r="38" ht="43.5" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>Compute</t>
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>VPN</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>SsmMessagesEndpoint</t>
+          <t>SamlProvider</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPCEndpoint</t>
+          <t>AWS::IAM::SAMLProvider</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>com.amazonaws.eu-central-1.ssmmessages</t>
+          <t>hmsg-rac-prd-clientvpn-saml</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>Interface · DbSubnetA · private DNS</t>
+          <t>Entra ID Federation Metadata XML</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -2033,34 +2029,34 @@
       <c r="G38" s="8" t="inlineStr"/>
     </row>
     <row r="39" ht="43.5" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>Compute</t>
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>VPN</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Ec2MessagesEndpoint</t>
+          <t>AcmCertificate</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPCEndpoint</t>
+          <t>AWS::CertificateManager::Certificate</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>com.amazonaws.eu-central-1.ec2messages</t>
+          <t>vpn.hmg-racing.com</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>Interface · DbSubnetA · private DNS</t>
+          <t>Public DNS validation (hosted zone)</t>
         </is>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CreateAcmCertHostedZone</t>
         </is>
       </c>
       <c r="G39" s="10" t="inlineStr"/>
@@ -2073,27 +2069,27 @@
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>SamlProvider</t>
+          <t>AcmCertificateManual</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>AWS::IAM::SAMLProvider</t>
+          <t>AWS::CertificateManager::Certificate</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-clientvpn-saml</t>
+          <t>vpn.hmg-racing.com</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Entra ID Federation Metadata XML</t>
+          <t>Public DNS validation (manual CNAME)</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CreateAcmCertManual</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr"/>
@@ -2106,27 +2102,27 @@
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>AcmCertificate</t>
+          <t>ClientVpnLogGroup</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>AWS::CertificateManager::Certificate</t>
+          <t>AWS::Logs::LogGroup</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>vpn.hmg-racing.com</t>
+          <t>hmsg-rac-prd-clientvpn-logs</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
-          <t>Public DNS validation (hosted zone)</t>
+          <t>CloudWatch · 90 day retention</t>
         </is>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
-          <t>CreateAcmCertHostedZone</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G41" s="10" t="inlineStr"/>
@@ -2139,27 +2135,27 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>AcmCertificateManual</t>
+          <t>ClientVpnEndpoint</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>AWS::CertificateManager::Certificate</t>
+          <t>AWS::EC2::ClientVpnEndpoint</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>vpn.hmg-racing.com</t>
+          <t>hmsg-rac-prd-clientvpn-ec1</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Public DNS validation (manual CNAME)</t>
+          <t>CIDR 10.200.0.0/22 · SAML federation · UDP 443 · split tunnel</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
-          <t>CreateAcmCertManual</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G42" s="8" t="inlineStr"/>
@@ -2172,22 +2168,22 @@
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>ClientVpnLogGroup</t>
+          <t>ClientVpnAssocPriA</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>AWS::Logs::LogGroup</t>
+          <t>AWS::EC2::ClientVpnTargetNetworkAssociation</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-clientvpn-logs</t>
+          <t>pri-a association</t>
         </is>
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>CloudWatch · 90 day retention</t>
+          <t>Target network PriSubnetA</t>
         </is>
       </c>
       <c r="F43" s="10" t="inlineStr">
@@ -2205,22 +2201,22 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>ClientVpnEndpoint</t>
+          <t>ClientVpnAssocPriC</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::ClientVpnEndpoint</t>
+          <t>AWS::EC2::ClientVpnTargetNetworkAssociation</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-clientvpn-ec1</t>
+          <t>pri-c association</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>CIDR 10.200.0.0/22 · SAML federation · UDP 443 · split tunnel</t>
+          <t>Target network PriSubnetC</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -2238,22 +2234,22 @@
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>ClientVpnAssocPriA</t>
+          <t>ClientVpnRouteVpc</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::ClientVpnTargetNetworkAssociation</t>
+          <t>AWS::EC2::ClientVpnRoute</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>pri-a association</t>
+          <t>route → VPC /24</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>Target network PriSubnetA</t>
+          <t>Via PriSubnetA association</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
@@ -2271,22 +2267,22 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>ClientVpnAssocPriC</t>
+          <t>ClientVpnAuthRule</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::ClientVpnTargetNetworkAssociation</t>
+          <t>AWS::EC2::ClientVpnAuthorizationRule</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>pri-c association</t>
+          <t>authorize all groups</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>Target network PriSubnetC</t>
+          <t>TargetNetworkCidr = VPC /24</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -2304,27 +2300,27 @@
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>ClientVpnRouteVpc</t>
+          <t>CustomerGateway</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::ClientVpnRoute</t>
+          <t>AWS::EC2::CustomerGateway</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>route → VPC /24</t>
+          <t>hmsg-rac-prd-cgw-ec1</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>Via PriSubnetA association</t>
+          <t>ipsec.1 · BGP ASN 65000 · public IP from client</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CreateSiteToSiteVpn</t>
         </is>
       </c>
       <c r="G47" s="10" t="inlineStr"/>
@@ -2337,27 +2333,27 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>ClientVpnAuthRule</t>
+          <t>VpnGateway</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::ClientVpnAuthorizationRule</t>
+          <t>AWS::EC2::VPNGateway</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>authorize all groups</t>
+          <t>hmsg-rac-prd-vgw-ec1</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>TargetNetworkCidr = VPC /24</t>
+          <t>ipsec.1 · Amazon side ASN 64512</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CreateSiteToSiteVpn</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr"/>
@@ -2370,22 +2366,22 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>CustomerGateway</t>
+          <t>VpcVgwAttachment</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::CustomerGateway</t>
+          <t>AWS::EC2::VPCGatewayAttachment</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-cgw-ec1</t>
+          <t>VPC ↔ VGW</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>ipsec.1 · BGP ASN 65000 · public IP from client</t>
+          <t>Attachment</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr">
@@ -2403,22 +2399,22 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>VpnGateway</t>
+          <t>VpnConnection</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPNGateway</t>
+          <t>AWS::EC2::VPNConnection</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-vgw-ec1</t>
+          <t>hmsg-rac-prd-vpn-conn-ec1</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>ipsec.1 · Amazon side ASN 64512</t>
+          <t>static routes only · 2 tunnels</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -2436,22 +2432,22 @@
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>VpcVgwAttachment</t>
+          <t>VpnConnectionRouteOnPrem</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPCGatewayAttachment</t>
+          <t>AWS::EC2::VPNConnectionRoute</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>VPC ↔ VGW</t>
+          <t>on-prem route</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>Attachment</t>
+          <t>Destination = OnPremCidr</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr">
@@ -2469,22 +2465,22 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>VpnConnection</t>
+          <t>VpnPropagationPri</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPNConnection</t>
+          <t>AWS::EC2::VPNGatewayRoutePropagation</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-vpn-conn-ec1</t>
+          <t>propagate → pri rtb</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>static routes only · 2 tunnels</t>
+          <t>VGW propagation</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
@@ -2502,22 +2498,22 @@
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>VpnConnectionRouteOnPrem</t>
+          <t>VpnPropagationDb</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPNConnectionRoute</t>
+          <t>AWS::EC2::VPNGatewayRoutePropagation</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>on-prem route</t>
+          <t>propagate → db rtb</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>Destination = OnPremCidr</t>
+          <t>VGW propagation</t>
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr">
@@ -2527,74 +2523,8 @@
       </c>
       <c r="G53" s="10" t="inlineStr"/>
     </row>
-    <row r="54" ht="43.5" customHeight="1">
-      <c r="A54" s="15" t="inlineStr">
-        <is>
-          <t>VPN</t>
-        </is>
-      </c>
-      <c r="B54" s="8" t="inlineStr">
-        <is>
-          <t>VpnPropagationPri</t>
-        </is>
-      </c>
-      <c r="C54" s="8" t="inlineStr">
-        <is>
-          <t>AWS::EC2::VPNGatewayRoutePropagation</t>
-        </is>
-      </c>
-      <c r="D54" s="8" t="inlineStr">
-        <is>
-          <t>propagate → pri rtb</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>VGW propagation</t>
-        </is>
-      </c>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>CreateSiteToSiteVpn</t>
-        </is>
-      </c>
-      <c r="G54" s="8" t="inlineStr"/>
-    </row>
-    <row r="55" ht="43.5" customHeight="1">
-      <c r="A55" s="16" t="inlineStr">
-        <is>
-          <t>VPN</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t>VpnPropagationDb</t>
-        </is>
-      </c>
-      <c r="C55" s="10" t="inlineStr">
-        <is>
-          <t>AWS::EC2::VPNGatewayRoutePropagation</t>
-        </is>
-      </c>
-      <c r="D55" s="10" t="inlineStr">
-        <is>
-          <t>propagate → db rtb</t>
-        </is>
-      </c>
-      <c r="E55" s="10" t="inlineStr">
-        <is>
-          <t>VGW propagation</t>
-        </is>
-      </c>
-      <c r="F55" s="10" t="inlineStr">
-        <is>
-          <t>CreateSiteToSiteVpn</t>
-        </is>
-      </c>
-      <c r="G55" s="10" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G55"/>
+  <autoFilter ref="A1:G53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -3166,7 +3096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3267,63 +3197,59 @@
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>FlowLogBucket</t>
+          <t>SysadmSecretArn</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>S3 bucket</t>
+          <t>Secrets Manager ARN</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>VPC flow logs</t>
+          <t>sysadm password</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>SysadmSecretArn</t>
+          <t>ServerCertificateArn</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Secrets Manager ARN</t>
+          <t>ACM certificate ARN</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>sysadm password</t>
+          <t>Client VPN server cert</t>
         </is>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>ServerCertificateArn</t>
+          <t>SamlProviderArn</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>ACM certificate ARN</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Client VPN server cert</t>
-        </is>
-      </c>
+          <t>IAM SAML provider ARN</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr"/>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
-          <t>SamlProviderArn</t>
+          <t>ClientVpnEndpointId</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>IAM SAML provider ARN</t>
+          <t>Endpoint ID</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr"/>
@@ -3331,12 +3257,12 @@
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>ClientVpnEndpointId</t>
+          <t>ClientVpnLogGroup</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Endpoint ID</t>
+          <t>CloudWatch log group</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr"/>
@@ -3344,69 +3270,56 @@
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="17" t="inlineStr">
         <is>
-          <t>ClientVpnLogGroup</t>
+          <t>CustomerGatewayId</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>CloudWatch log group</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr"/>
+          <t>CGW ID</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Only with S2S VPN</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>CustomerGatewayId</t>
+          <t>VpnConnectionId</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>CGW ID</t>
+          <t>VPN connection ID</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Only with S2S VPN</t>
+          <t>Tunnel config source</t>
         </is>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>VpnConnectionId</t>
+          <t>SiteToSiteVpnDeployed</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>VPN connection ID</t>
+          <t>true / false</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Tunnel config source</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>SiteToSiteVpnDeployed</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>true / false</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
           <t>Indicator</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C15"/>
+  <autoFilter ref="A1:C14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Drop explicit ClientVpnRouteVpc: AWS auto-adds the VPC CIDR route on subnet association
- ClientVpnTargetNetworkAssociation auto-creates a route to VpcCidr
  (Origin: associate-target-network); explicit ClientVpnRoute to the same
  CIDR failed the deploy with InvalidClientVpnDuplicateRoute (Route already exists)
- Remove resource from template + resource-inventory generator row
- Regression: also clean up ROLLBACK_FAILED leftovers from the failed run
</commit_message>
<xml_diff>
--- a/deliverables/AWS-Infrastructure-Resource-Inventory.xlsx
+++ b/deliverables/AWS-Infrastructure-Resource-Inventory.xlsx
@@ -16,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users &amp; Permissions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resource Inventory'!$A$1:$G$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Resource Inventory'!$A$1:$G$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Parameters'!$A$1:$D$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Conditions'!$A$1:$C$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Outputs'!$A$1:$C$14</definedName>
@@ -665,7 +665,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>19 August 2026</t>
+          <t>20 August 2026</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2234,22 +2234,22 @@
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>ClientVpnRouteVpc</t>
+          <t>ClientVpnAuthRule</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::ClientVpnRoute</t>
+          <t>AWS::EC2::ClientVpnAuthorizationRule</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>route → VPC /24</t>
+          <t>authorize all groups</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>Via PriSubnetA association</t>
+          <t>TargetNetworkCidr = VPC /24</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
@@ -2267,27 +2267,27 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>ClientVpnAuthRule</t>
+          <t>CustomerGateway</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::ClientVpnAuthorizationRule</t>
+          <t>AWS::EC2::CustomerGateway</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>authorize all groups</t>
+          <t>hmsg-rac-prd-cgw-ec1</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>TargetNetworkCidr = VPC /24</t>
+          <t>ipsec.1 · BGP ASN 65000 · public IP from client</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CreateSiteToSiteVpn</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr"/>
@@ -2300,22 +2300,22 @@
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>CustomerGateway</t>
+          <t>VpnGateway</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::CustomerGateway</t>
+          <t>AWS::EC2::VPNGateway</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-cgw-ec1</t>
+          <t>hmsg-rac-prd-vgw-ec1</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>ipsec.1 · BGP ASN 65000 · public IP from client</t>
+          <t>ipsec.1 · Amazon side ASN 64512</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
@@ -2333,22 +2333,22 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>VpnGateway</t>
+          <t>VpcVgwAttachment</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPNGateway</t>
+          <t>AWS::EC2::VPCGatewayAttachment</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-vgw-ec1</t>
+          <t>VPC ↔ VGW</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>ipsec.1 · Amazon side ASN 64512</t>
+          <t>Attachment</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -2366,22 +2366,22 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>VpcVgwAttachment</t>
+          <t>VpnConnection</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPCGatewayAttachment</t>
+          <t>AWS::EC2::VPNConnection</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>VPC ↔ VGW</t>
+          <t>hmsg-rac-prd-vpn-conn-ec1</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
         <is>
-          <t>Attachment</t>
+          <t>static routes only · 2 tunnels</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr">
@@ -2399,22 +2399,22 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>VpnConnection</t>
+          <t>VpnConnectionRouteOnPrem</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPNConnection</t>
+          <t>AWS::EC2::VPNConnectionRoute</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>hmsg-rac-prd-vpn-conn-ec1</t>
+          <t>on-prem route</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>static routes only · 2 tunnels</t>
+          <t>Destination = OnPremCidr</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -2432,22 +2432,22 @@
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>VpnConnectionRouteOnPrem</t>
+          <t>VpnPropagationPri</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>AWS::EC2::VPNConnectionRoute</t>
+          <t>AWS::EC2::VPNGatewayRoutePropagation</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>on-prem route</t>
+          <t>propagate → pri rtb</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr">
         <is>
-          <t>Destination = OnPremCidr</t>
+          <t>VGW propagation</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>VpnPropagationPri</t>
+          <t>VpnPropagationDb</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>propagate → pri rtb</t>
+          <t>propagate → db rtb</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
@@ -2490,41 +2490,8 @@
       </c>
       <c r="G52" s="8" t="inlineStr"/>
     </row>
-    <row r="53" ht="43.5" customHeight="1">
-      <c r="A53" s="16" t="inlineStr">
-        <is>
-          <t>VPN</t>
-        </is>
-      </c>
-      <c r="B53" s="10" t="inlineStr">
-        <is>
-          <t>VpnPropagationDb</t>
-        </is>
-      </c>
-      <c r="C53" s="10" t="inlineStr">
-        <is>
-          <t>AWS::EC2::VPNGatewayRoutePropagation</t>
-        </is>
-      </c>
-      <c r="D53" s="10" t="inlineStr">
-        <is>
-          <t>propagate → db rtb</t>
-        </is>
-      </c>
-      <c r="E53" s="10" t="inlineStr">
-        <is>
-          <t>VGW propagation</t>
-        </is>
-      </c>
-      <c r="F53" s="10" t="inlineStr">
-        <is>
-          <t>CreateSiteToSiteVpn</t>
-        </is>
-      </c>
-      <c r="G53" s="10" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G53"/>
+  <autoFilter ref="A1:G52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>